<commit_message>
Remove em-dashes repo-wide; fix mandate-B offline fixture selection
Replace all em-dash characters with plain hyphens across docs, configs,
source comments/docstrings, and generated deliverables/outputs, then
regenerate the Jatayu and Outreach outputs so generated files stay
consistent with the fixed source templates (ranking rationale,
outreach positioning copy, etc.).

While regenerating, found and fixed a latent bug: offline runs always
defaulted to Mandate A's fixtures regardless of which mandate config
was passed, so Mandate B's run produced zero results. Added
Settings.autoselect_fixtures() to pick the matching fixtures file per
mandate id, used by both `jatayu run` and `jatayu preview`.
</commit_message>
<xml_diff>
--- a/jatayu/deliverables/mandate_a/top10_shortlist.xlsx
+++ b/jatayu/deliverables/mandate_a/top10_shortlist.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -870,7 +870,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
         <v>95</v>
       </c>
       <c r="M9" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>